<commit_message>
Fix relic column widths
</commit_message>
<xml_diff>
--- a/sts2_cards.xlsx
+++ b/sts2_cards.xlsx
@@ -22665,11 +22665,11 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
-    <col width="25" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="80" customWidth="1" min="6" max="6"/>
+    <col width="60" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">

</xml_diff>

<commit_message>
Add spacer column before relic description
</commit_message>
<xml_diff>
--- a/sts2_cards.xlsx
+++ b/sts2_cards.xlsx
@@ -22661,7 +22661,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F218"/>
+  <dimension ref="A1:G218"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -22669,7 +22669,8 @@
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="60" customWidth="1" min="6" max="6"/>
+    <col width="5" customWidth="1" min="6" max="6"/>
+    <col width="55" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -22698,7 +22699,8 @@
           <t>Win%</t>
         </is>
       </c>
-      <c r="F1" s="7" t="inlineStr">
+      <c r="F1" s="7" t="inlineStr"/>
+      <c r="G1" s="7" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
@@ -22724,7 +22726,8 @@
       <c r="E2" t="n">
         <v>19.5</v>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="inlineStr">
         <is>
           <t>At the start of each combat, draw 2 additional cards.</t>
         </is>
@@ -22750,7 +22753,8 @@
       <c r="E3" t="n">
         <v>26.7</v>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="inlineStr">
         <is>
           <t>At the start of each combat, Channel 1 Lightning.</t>
         </is>
@@ -22776,7 +22780,8 @@
       <c r="E4" t="n">
         <v>21.4</v>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr">
         <is>
           <t>At the end of combat, heal 6 HP.</t>
         </is>
@@ -22802,7 +22807,8 @@
       <c r="E5" t="n">
         <v>52.2</v>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="inlineStr">
         <is>
           <t>Upon pickup, Upgrade 2 random Skills.</t>
         </is>
@@ -22828,7 +22834,8 @@
       <c r="E6" t="n">
         <v>22.7</v>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="F6" t="inlineStr"/>
+      <c r="G6" t="inlineStr">
         <is>
           <t>Upon pickup, lose all Gold and choose 1 of 2 packs of cards.</t>
         </is>
@@ -22854,7 +22861,8 @@
       <c r="E7" t="n">
         <v>52.4</v>
       </c>
-      <c r="F7" t="inlineStr">
+      <c r="F7" t="inlineStr"/>
+      <c r="G7" t="inlineStr">
         <is>
           <t>At the start of each combat, draw 2 additional cards.</t>
         </is>
@@ -22880,7 +22888,8 @@
       <c r="E8" t="n">
         <v>57.9</v>
       </c>
-      <c r="F8" t="inlineStr">
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="inlineStr">
         <is>
           <t>Upon pickup, raise your Max HP by 7.</t>
         </is>
@@ -22906,7 +22915,8 @@
       <c r="E9" t="n">
         <v>44.4</v>
       </c>
-      <c r="F9" t="inlineStr">
+      <c r="F9" t="inlineStr"/>
+      <c r="G9" t="inlineStr">
         <is>
           <t>At the start of your turn, Summon 1.</t>
         </is>
@@ -22932,7 +22942,8 @@
       <c r="E10" t="n">
         <v>66.7</v>
       </c>
-      <c r="F10" t="inlineStr">
+      <c r="F10" t="inlineStr"/>
+      <c r="G10" t="inlineStr">
         <is>
           <t>Upon pickup, Upgrade 2 random Attacks.</t>
         </is>
@@ -22958,7 +22969,8 @@
       <c r="E11" t="n">
         <v>47.1</v>
       </c>
-      <c r="F11" t="inlineStr">
+      <c r="F11" t="inlineStr"/>
+      <c r="G11" t="inlineStr">
         <is>
           <t>Whenever you Rest, procure a random potion.</t>
         </is>
@@ -22984,7 +22996,8 @@
       <c r="E12" t="n">
         <v>64.7</v>
       </c>
-      <c r="F12" t="inlineStr">
+      <c r="F12" t="inlineStr"/>
+      <c r="G12" t="inlineStr">
         <is>
           <t>Whenever you shuffle your Draw Pile, draw a card.</t>
         </is>
@@ -23010,7 +23023,8 @@
       <c r="E13" t="n">
         <v>6.2</v>
       </c>
-      <c r="F13" t="inlineStr">
+      <c r="F13" t="inlineStr"/>
+      <c r="G13" t="inlineStr">
         <is>
           <t>Upon pickup, Transform 1 of your Strikes and 1 of your Defends.</t>
         </is>
@@ -23036,7 +23050,8 @@
       <c r="E14" t="n">
         <v>50</v>
       </c>
-      <c r="F14" t="inlineStr">
+      <c r="F14" t="inlineStr"/>
+      <c r="G14" t="inlineStr">
         <is>
           <t>If you end your turn without Block, gain 6 Block.</t>
         </is>
@@ -23062,7 +23077,8 @@
       <c r="E15" t="n">
         <v>50</v>
       </c>
-      <c r="F15" t="inlineStr">
+      <c r="F15" t="inlineStr"/>
+      <c r="G15" t="inlineStr">
         <is>
           <t>Every time you play 3 Attacks in a single turn, deal 6 damage to a random enemy.</t>
         </is>
@@ -23088,7 +23104,8 @@
       <c r="E16" t="n">
         <v>43.8</v>
       </c>
-      <c r="F16" t="inlineStr">
+      <c r="F16" t="inlineStr"/>
+      <c r="G16" t="inlineStr">
         <is>
           <t>Start each combat with an additional 1 energy.</t>
         </is>
@@ -23114,7 +23131,8 @@
       <c r="E17" t="n">
         <v>12.5</v>
       </c>
-      <c r="F17" t="inlineStr">
+      <c r="F17" t="inlineStr"/>
+      <c r="G17" t="inlineStr">
         <is>
           <t>The first 3 card rewards you see are Upgraded.</t>
         </is>
@@ -23140,7 +23158,8 @@
       <c r="E18" t="n">
         <v>60</v>
       </c>
-      <c r="F18" t="inlineStr">
+      <c r="F18" t="inlineStr"/>
+      <c r="G18" t="inlineStr">
         <is>
           <t>At the start of each combat, heal 2 HP.</t>
         </is>
@@ -23166,7 +23185,8 @@
       <c r="E19" t="n">
         <v>66.7</v>
       </c>
-      <c r="F19" t="inlineStr">
+      <c r="F19" t="inlineStr"/>
+      <c r="G19" t="inlineStr">
         <is>
           <t>Whenever you enter a Rest Site, start the next combat with an additional 2 energy.</t>
         </is>
@@ -23192,7 +23212,8 @@
       <c r="E20" t="n">
         <v>46.7</v>
       </c>
-      <c r="F20" t="inlineStr">
+      <c r="F20" t="inlineStr"/>
+      <c r="G20" t="inlineStr">
         <is>
           <t>Upon pickup, remove 2 cards from your Deck.</t>
         </is>
@@ -23218,7 +23239,8 @@
       <c r="E21" t="n">
         <v>53.3</v>
       </c>
-      <c r="F21" t="inlineStr">
+      <c r="F21" t="inlineStr"/>
+      <c r="G21" t="inlineStr">
         <is>
           <t>Start each combat with 1 Strength.</t>
         </is>
@@ -23244,7 +23266,8 @@
       <c r="E22" t="n">
         <v>40</v>
       </c>
-      <c r="F22" t="inlineStr">
+      <c r="F22" t="inlineStr"/>
+      <c r="G22" t="inlineStr">
         <is>
           <t>Start each combat with 10 Block.</t>
         </is>
@@ -23270,7 +23293,8 @@
       <c r="E23" t="n">
         <v>50</v>
       </c>
-      <c r="F23" t="inlineStr">
+      <c r="F23" t="inlineStr"/>
+      <c r="G23" t="inlineStr">
         <is>
           <t>At the start of each combat, gain 4 Plating.</t>
         </is>
@@ -23296,7 +23320,8 @@
       <c r="E24" t="n">
         <v>28.6</v>
       </c>
-      <c r="F24" t="inlineStr">
+      <c r="F24" t="inlineStr"/>
+      <c r="G24" t="inlineStr">
         <is>
           <t>Whenever you Rest, heal an additional 15 HP.</t>
         </is>
@@ -23322,7 +23347,8 @@
       <c r="E25" t="n">
         <v>61.5</v>
       </c>
-      <c r="F25" t="inlineStr">
+      <c r="F25" t="inlineStr"/>
+      <c r="G25" t="inlineStr">
         <is>
           <t>Start each combat with 3 Thorns.</t>
         </is>
@@ -23348,7 +23374,8 @@
       <c r="E26" t="n">
         <v>53.8</v>
       </c>
-      <c r="F26" t="inlineStr">
+      <c r="F26" t="inlineStr"/>
+      <c r="G26" t="inlineStr">
         <is>
           <t>Every 3 turns, gain 1 energy.</t>
         </is>
@@ -23374,7 +23401,8 @@
       <c r="E27" t="n">
         <v>38.5</v>
       </c>
-      <c r="F27" t="inlineStr">
+      <c r="F27" t="inlineStr"/>
+      <c r="G27" t="inlineStr">
         <is>
           <t>The first time you play a Power each combat, gain 6 Block.</t>
         </is>
@@ -23400,7 +23428,8 @@
       <c r="E28" t="n">
         <v>16.7</v>
       </c>
-      <c r="F28" t="inlineStr">
+      <c r="F28" t="inlineStr"/>
+      <c r="G28" t="inlineStr">
         <is>
           <t>At the start of each combat, gain 3 Star.</t>
         </is>
@@ -23426,7 +23455,8 @@
       <c r="E29" t="n">
         <v>75</v>
       </c>
-      <c r="F29" t="inlineStr">
+      <c r="F29" t="inlineStr"/>
+      <c r="G29" t="inlineStr">
         <is>
           <t>For every 5 cards in your Deck, heal 3 HP whenever you enter a Rest Site.</t>
         </is>
@@ -23452,7 +23482,8 @@
       <c r="E30" t="n">
         <v>91.7</v>
       </c>
-      <c r="F30" t="inlineStr">
+      <c r="F30" t="inlineStr"/>
+      <c r="G30" t="inlineStr">
         <is>
           <t>If you did not play any Attacks during your turn, gain 4 Block.</t>
         </is>
@@ -23478,7 +23509,8 @@
       <c r="E31" t="n">
         <v>16.7</v>
       </c>
-      <c r="F31" t="inlineStr">
+      <c r="F31" t="inlineStr"/>
+      <c r="G31" t="inlineStr">
         <is>
           <t>Upon pickup, obtain a random Rare Card to add to your Deck.</t>
         </is>
@@ -23504,7 +23536,8 @@
       <c r="E32" t="n">
         <v>41.7</v>
       </c>
-      <c r="F32" t="inlineStr">
+      <c r="F32" t="inlineStr"/>
+      <c r="G32" t="inlineStr">
         <is>
           <t>Regular enemy combats are no longer encountered in ? rooms.</t>
         </is>
@@ -23530,7 +23563,8 @@
       <c r="E33" t="n">
         <v>41.7</v>
       </c>
-      <c r="F33" t="inlineStr">
+      <c r="F33" t="inlineStr"/>
+      <c r="G33" t="inlineStr">
         <is>
           <t>Gain 20% additional Gold.</t>
         </is>
@@ -23556,7 +23590,8 @@
       <c r="E34" t="n">
         <v>75</v>
       </c>
-      <c r="F34" t="inlineStr">
+      <c r="F34" t="inlineStr"/>
+      <c r="G34" t="inlineStr">
         <is>
           <t>Start each combat with 1 Dexterity.</t>
         </is>
@@ -23582,7 +23617,8 @@
       <c r="E35" t="n">
         <v>66.7</v>
       </c>
-      <c r="F35" t="inlineStr">
+      <c r="F35" t="inlineStr"/>
+      <c r="G35" t="inlineStr">
         <is>
           <t>Every time you play 3 Skills in a single turn, deal 5 damage to ALL enemies.</t>
         </is>
@@ -23608,7 +23644,8 @@
       <c r="E36" t="n">
         <v>75</v>
       </c>
-      <c r="F36" t="inlineStr">
+      <c r="F36" t="inlineStr"/>
+      <c r="G36" t="inlineStr">
         <is>
           <t>At the start of each Boss combat, heal 25 HP.</t>
         </is>
@@ -23634,7 +23671,8 @@
       <c r="E37" t="n">
         <v>41.7</v>
       </c>
-      <c r="F37" t="inlineStr">
+      <c r="F37" t="inlineStr"/>
+      <c r="G37" t="inlineStr">
         <is>
           <t>At the start of your 2nd turn, gain 14 Block.</t>
         </is>
@@ -23660,7 +23698,8 @@
       <c r="E38" t="n">
         <v>63.6</v>
       </c>
-      <c r="F38" t="inlineStr">
+      <c r="F38" t="inlineStr"/>
+      <c r="G38" t="inlineStr">
         <is>
           <t>Upon pickup, gain 2 potion slots.</t>
         </is>
@@ -23686,7 +23725,8 @@
       <c r="E39" t="n">
         <v>36.4</v>
       </c>
-      <c r="F39" t="inlineStr">
+      <c r="F39" t="inlineStr"/>
+      <c r="G39" t="inlineStr">
         <is>
           <t>At the start of each combat, gain 8 Vigor.</t>
         </is>
@@ -23712,7 +23752,8 @@
       <c r="E40" t="n">
         <v>90.90000000000001</v>
       </c>
-      <c r="F40" t="inlineStr">
+      <c r="F40" t="inlineStr"/>
+      <c r="G40" t="inlineStr">
         <is>
           <t>At the start of your turn, deal 3 damage to ALL enemies.</t>
         </is>
@@ -23738,7 +23779,8 @@
       <c r="E41" t="n">
         <v>54.5</v>
       </c>
-      <c r="F41" t="inlineStr">
+      <c r="F41" t="inlineStr"/>
+      <c r="G41" t="inlineStr">
         <is>
           <t>Whenever you enter a shop room, heal 15 HP.</t>
         </is>
@@ -23764,7 +23806,8 @@
       <c r="E42" t="n">
         <v>54.5</v>
       </c>
-      <c r="F42" t="inlineStr">
+      <c r="F42" t="inlineStr"/>
+      <c r="G42" t="inlineStr">
         <is>
           <t>The first time you lose HP each combat, draw 3 cards.</t>
         </is>
@@ -23790,7 +23833,8 @@
       <c r="E43" t="n">
         <v>36.4</v>
       </c>
-      <c r="F43" t="inlineStr">
+      <c r="F43" t="inlineStr"/>
+      <c r="G43" t="inlineStr">
         <is>
           <t>Every 5 cards you add to your Deck, heal 15 HP.</t>
         </is>
@@ -23816,7 +23860,8 @@
       <c r="E44" t="n">
         <v>20</v>
       </c>
-      <c r="F44" t="inlineStr">
+      <c r="F44" t="inlineStr"/>
+      <c r="G44" t="inlineStr">
         <is>
           <t>Upon pickup, receive Greed. Gain 333 Gold.</t>
         </is>
@@ -23842,7 +23887,8 @@
       <c r="E45" t="n">
         <v>70</v>
       </c>
-      <c r="F45" t="inlineStr">
+      <c r="F45" t="inlineStr"/>
+      <c r="G45" t="inlineStr">
         <is>
           <t>The first Hand you draw each combat is Upgraded.</t>
         </is>
@@ -23868,7 +23914,8 @@
       <c r="E46" t="n">
         <v>70</v>
       </c>
-      <c r="F46" t="inlineStr">
+      <c r="F46" t="inlineStr"/>
+      <c r="G46" t="inlineStr">
         <is>
           <t>Cards containing Strike deal 3 additional damage.</t>
         </is>
@@ -23894,7 +23941,8 @@
       <c r="E47" t="n">
         <v>50</v>
       </c>
-      <c r="F47" t="inlineStr">
+      <c r="F47" t="inlineStr"/>
+      <c r="G47" t="inlineStr">
         <is>
           <t>The first time you gain Block from a card each combat, double the amount gained.</t>
         </is>
@@ -23920,7 +23968,8 @@
       <c r="E48" t="n">
         <v>0</v>
       </c>
-      <c r="F48" t="inlineStr">
+      <c r="F48" t="inlineStr"/>
+      <c r="G48" t="inlineStr">
         <is>
           <t>At the start of each combat, apply 1 Vulnerable to ALL enemies.</t>
         </is>
@@ -23946,7 +23995,8 @@
       <c r="E49" t="n">
         <v>33.3</v>
       </c>
-      <c r="F49" t="inlineStr">
+      <c r="F49" t="inlineStr"/>
+      <c r="G49" t="inlineStr">
         <is>
           <t>At the start of each combat, apply 1 Weak to ALL enemies.</t>
         </is>
@@ -23972,7 +24022,8 @@
       <c r="E50" t="n">
         <v>44.4</v>
       </c>
-      <c r="F50" t="inlineStr">
+      <c r="F50" t="inlineStr"/>
+      <c r="G50" t="inlineStr">
         <is>
           <t>Enemies drop 10 additional Gold.</t>
         </is>
@@ -23998,7 +24049,8 @@
       <c r="E51" t="n">
         <v>33.3</v>
       </c>
-      <c r="F51" t="inlineStr">
+      <c r="F51" t="inlineStr"/>
+      <c r="G51" t="inlineStr">
         <is>
           <t>If you end a turn with at least 10 Block, deal 6 damage to a random enemy.</t>
         </is>
@@ -24024,7 +24076,8 @@
       <c r="E52" t="n">
         <v>77.8</v>
       </c>
-      <c r="F52" t="inlineStr">
+      <c r="F52" t="inlineStr"/>
+      <c r="G52" t="inlineStr">
         <is>
           <t>At the start of your 2nd turn, gain 2 energy.</t>
         </is>
@@ -24050,7 +24103,8 @@
       <c r="E53" t="n">
         <v>44.4</v>
       </c>
-      <c r="F53" t="inlineStr">
+      <c r="F53" t="inlineStr"/>
+      <c r="G53" t="inlineStr">
         <is>
           <t>At the start of each combat, deal 9 damage to ALL enemies.</t>
         </is>
@@ -24076,7 +24130,8 @@
       <c r="E54" t="n">
         <v>50</v>
       </c>
-      <c r="F54" t="inlineStr">
+      <c r="F54" t="inlineStr"/>
+      <c r="G54" t="inlineStr">
         <is>
           <t>Whenever you add a card that gains Block to your Deck, Enchant it with Nimble 2.</t>
         </is>
@@ -24102,7 +24157,8 @@
       <c r="E55" t="n">
         <v>37.5</v>
       </c>
-      <c r="F55" t="inlineStr">
+      <c r="F55" t="inlineStr"/>
+      <c r="G55" t="inlineStr">
         <is>
           <t>At the start of Boss combats, Upgrade 3 random cards.</t>
         </is>
@@ -24128,7 +24184,8 @@
       <c r="E56" t="n">
         <v>50</v>
       </c>
-      <c r="F56" t="inlineStr">
+      <c r="F56" t="inlineStr"/>
+      <c r="G56" t="inlineStr">
         <is>
           <t>Whenever you use a potion, gain 3 Strength this turn.</t>
         </is>
@@ -24154,7 +24211,8 @@
       <c r="E57" t="n">
         <v>50</v>
       </c>
-      <c r="F57" t="inlineStr">
+      <c r="F57" t="inlineStr"/>
+      <c r="G57" t="inlineStr">
         <is>
           <t>Every time you play 10 Attacks, gain 1 energy.</t>
         </is>
@@ -24180,7 +24238,8 @@
       <c r="E58" t="n">
         <v>37.5</v>
       </c>
-      <c r="F58" t="inlineStr">
+      <c r="F58" t="inlineStr"/>
+      <c r="G58" t="inlineStr">
         <is>
           <t>Unknown</t>
         </is>
@@ -24206,7 +24265,8 @@
       <c r="E59" t="n">
         <v>57.1</v>
       </c>
-      <c r="F59" t="inlineStr">
+      <c r="F59" t="inlineStr"/>
+      <c r="G59" t="inlineStr">
         <is>
           <t>Whenever you enter a ? room, heal 4 HP.</t>
         </is>
@@ -24232,7 +24292,8 @@
       <c r="E60" t="n">
         <v>28.6</v>
       </c>
-      <c r="F60" t="inlineStr">
+      <c r="F60" t="inlineStr"/>
+      <c r="G60" t="inlineStr">
         <is>
           <t>Whenever you add a card to your Deck, gain 15 Gold.</t>
         </is>
@@ -24258,7 +24319,8 @@
       <c r="E61" t="n">
         <v>71.40000000000001</v>
       </c>
-      <c r="F61" t="inlineStr">
+      <c r="F61" t="inlineStr"/>
+      <c r="G61" t="inlineStr">
         <is>
           <t>Upon pickup, obtain an Ancient Card.</t>
         </is>
@@ -24284,7 +24346,8 @@
       <c r="E62" t="n">
         <v>42.9</v>
       </c>
-      <c r="F62" t="inlineStr">
+      <c r="F62" t="inlineStr"/>
+      <c r="G62" t="inlineStr">
         <is>
           <t>Every 10th Attack you play deals double damage.</t>
         </is>
@@ -24310,7 +24373,8 @@
       <c r="E63" t="n">
         <v>42.9</v>
       </c>
-      <c r="F63" t="inlineStr">
+      <c r="F63" t="inlineStr"/>
+      <c r="G63" t="inlineStr">
         <is>
           <t>Upon pickup, remove 1 card from your Deck.</t>
         </is>
@@ -24336,7 +24400,8 @@
       <c r="E64" t="n">
         <v>28.6</v>
       </c>
-      <c r="F64" t="inlineStr">
+      <c r="F64" t="inlineStr"/>
+      <c r="G64" t="inlineStr">
         <is>
           <t>Whenever an enemy dies, gain 1 energy and draw 1 card.</t>
         </is>
@@ -24362,7 +24427,8 @@
       <c r="E65" t="n">
         <v>42.9</v>
       </c>
-      <c r="F65" t="inlineStr">
+      <c r="F65" t="inlineStr"/>
+      <c r="G65" t="inlineStr">
         <is>
           <t>Upon pickup, Upgrade 4 cards.</t>
         </is>
@@ -24388,7 +24454,8 @@
       <c r="E66" t="n">
         <v>57.1</v>
       </c>
-      <c r="F66" t="inlineStr">
+      <c r="F66" t="inlineStr"/>
+      <c r="G66" t="inlineStr">
         <is>
           <t>Whenever you play a Power, a random card in your Hand is free to play that turn.</t>
         </is>
@@ -24414,7 +24481,8 @@
       <c r="E67" t="n">
         <v>14.3</v>
       </c>
-      <c r="F67" t="inlineStr">
+      <c r="F67" t="inlineStr"/>
+      <c r="G67" t="inlineStr">
         <is>
           <t>Whenever you Rest, you may add a card to your Deck.</t>
         </is>
@@ -24440,7 +24508,8 @@
       <c r="E68" t="n">
         <v>42.9</v>
       </c>
-      <c r="F68" t="inlineStr">
+      <c r="F68" t="inlineStr"/>
+      <c r="G68" t="inlineStr">
         <is>
           <t>Upon pickup, Transform 1 card.</t>
         </is>
@@ -24466,7 +24535,8 @@
       <c r="E69" t="n">
         <v>50</v>
       </c>
-      <c r="F69" t="inlineStr">
+      <c r="F69" t="inlineStr"/>
+      <c r="G69" t="inlineStr">
         <is>
           <t>Every time you play 3 Attacks in a single turn, gain 4 Block.</t>
         </is>
@@ -24492,7 +24562,8 @@
       <c r="E70" t="n">
         <v>66.7</v>
       </c>
-      <c r="F70" t="inlineStr">
+      <c r="F70" t="inlineStr"/>
+      <c r="G70" t="inlineStr">
         <is>
           <t>At the end of your turn, gain 1 Block for each card in your Hand.</t>
         </is>
@@ -24518,7 +24589,8 @@
       <c r="E71" t="n">
         <v>50</v>
       </c>
-      <c r="F71" t="inlineStr">
+      <c r="F71" t="inlineStr"/>
+      <c r="G71" t="inlineStr">
         <is>
           <t>At the start of your 3rd turn, gain 18 Block.</t>
         </is>
@@ -24544,7 +24616,8 @@
       <c r="E72" t="n">
         <v>66.7</v>
       </c>
-      <c r="F72" t="inlineStr">
+      <c r="F72" t="inlineStr"/>
+      <c r="G72" t="inlineStr">
         <is>
           <t>Whenever you would lose HP, lose 1 less.</t>
         </is>
@@ -24570,7 +24643,8 @@
       <c r="E73" t="n">
         <v>66.7</v>
       </c>
-      <c r="F73" t="inlineStr">
+      <c r="F73" t="inlineStr"/>
+      <c r="G73" t="inlineStr">
         <is>
           <t>Each combat, the first time you play a card that Debuffs an enemy, double its effect.</t>
         </is>
@@ -24596,7 +24670,8 @@
       <c r="E74" t="n">
         <v>50</v>
       </c>
-      <c r="F74" t="inlineStr">
+      <c r="F74" t="inlineStr"/>
+      <c r="G74" t="inlineStr">
         <is>
           <t>Upon pickup, raise your Max HP by 10.</t>
         </is>
@@ -24622,7 +24697,8 @@
       <c r="E75" t="n">
         <v>83.3</v>
       </c>
-      <c r="F75" t="inlineStr">
+      <c r="F75" t="inlineStr"/>
+      <c r="G75" t="inlineStr">
         <is>
           <t>Start each combat with an additional 4 energy.</t>
         </is>
@@ -24648,7 +24724,8 @@
       <c r="E76" t="n">
         <v>66.7</v>
       </c>
-      <c r="F76" t="inlineStr">
+      <c r="F76" t="inlineStr"/>
+      <c r="G76" t="inlineStr">
         <is>
           <t>Start each combat with 1 Focus.</t>
         </is>
@@ -24674,7 +24751,8 @@
       <c r="E77" t="n">
         <v>33.3</v>
       </c>
-      <c r="F77" t="inlineStr">
+      <c r="F77" t="inlineStr"/>
+      <c r="G77" t="inlineStr">
         <is>
           <t>Upon pickup, choose 1 of 2 Colorless cards to add to your Deck.</t>
         </is>
@@ -24700,7 +24778,8 @@
       <c r="E78" t="n">
         <v>50</v>
       </c>
-      <c r="F78" t="inlineStr">
+      <c r="F78" t="inlineStr"/>
+      <c r="G78" t="inlineStr">
         <is>
           <t>The first time you play an Attack, Skill, and Power each turn, gain 1 Strength and 1 Dexterity.</t>
         </is>
@@ -24726,7 +24805,8 @@
       <c r="E79" t="n">
         <v>100</v>
       </c>
-      <c r="F79" t="inlineStr">
+      <c r="F79" t="inlineStr"/>
+      <c r="G79" t="inlineStr">
         <is>
           <t>Upon pickup, gain 999 Gold.</t>
         </is>
@@ -24752,7 +24832,8 @@
       <c r="E80" t="n">
         <v>83.3</v>
       </c>
-      <c r="F80" t="inlineStr">
+      <c r="F80" t="inlineStr"/>
+      <c r="G80" t="inlineStr">
         <is>
           <t>Whenever you play a Power, draw 1 card.</t>
         </is>
@@ -24778,7 +24859,8 @@
       <c r="E81" t="n">
         <v>60</v>
       </c>
-      <c r="F81" t="inlineStr">
+      <c r="F81" t="inlineStr"/>
+      <c r="G81" t="inlineStr">
         <is>
           <t>Every time you play 3 Attacks in a single turn, gain 1 Strength.</t>
         </is>
@@ -24804,7 +24886,8 @@
       <c r="E82" t="n">
         <v>80</v>
       </c>
-      <c r="F82" t="inlineStr">
+      <c r="F82" t="inlineStr"/>
+      <c r="G82" t="inlineStr">
         <is>
           <t>When you would die, heal to 50% of your Max HP instead.</t>
         </is>
@@ -24830,7 +24913,8 @@
       <c r="E83" t="n">
         <v>80</v>
       </c>
-      <c r="F83" t="inlineStr">
+      <c r="F83" t="inlineStr"/>
+      <c r="G83" t="inlineStr">
         <is>
           <t>You cannot lose more than 20 HP in a single turn.</t>
         </is>
@@ -24856,7 +24940,8 @@
       <c r="E84" t="n">
         <v>40</v>
       </c>
-      <c r="F84" t="inlineStr">
+      <c r="F84" t="inlineStr"/>
+      <c r="G84" t="inlineStr">
         <is>
           <t>Upon pickup, Upgrade a card.</t>
         </is>
@@ -24882,7 +24967,8 @@
       <c r="E85" t="n">
         <v>60</v>
       </c>
-      <c r="F85" t="inlineStr">
+      <c r="F85" t="inlineStr"/>
+      <c r="G85" t="inlineStr">
         <is>
           <t>Up to 10 Block persists across turns.</t>
         </is>
@@ -24908,7 +24994,8 @@
       <c r="E86" t="n">
         <v>80</v>
       </c>
-      <c r="F86" t="inlineStr">
+      <c r="F86" t="inlineStr"/>
+      <c r="G86" t="inlineStr">
         <is>
           <t>At the start of your 3rd turn, gain 3 energy.</t>
         </is>
@@ -24934,7 +25021,8 @@
       <c r="E87" t="n">
         <v>60</v>
       </c>
-      <c r="F87" t="inlineStr">
+      <c r="F87" t="inlineStr"/>
+      <c r="G87" t="inlineStr">
         <is>
           <t>Every time you play 10 Skills, gain 7 Block.</t>
         </is>
@@ -24960,7 +25048,8 @@
       <c r="E88" t="n">
         <v>60</v>
       </c>
-      <c r="F88" t="inlineStr">
+      <c r="F88" t="inlineStr"/>
+      <c r="G88" t="inlineStr">
         <is>
           <t>Upon pickup, Enchant all Defends with Goopy.</t>
         </is>
@@ -24986,7 +25075,8 @@
       <c r="E89" t="n">
         <v>40</v>
       </c>
-      <c r="F89" t="inlineStr">
+      <c r="F89" t="inlineStr"/>
+      <c r="G89" t="inlineStr">
         <is>
           <t>You may choose any number of options at Rest Sites.</t>
         </is>
@@ -25012,7 +25102,8 @@
       <c r="E90" t="n">
         <v>20</v>
       </c>
-      <c r="F90" t="inlineStr">
+      <c r="F90" t="inlineStr"/>
+      <c r="G90" t="inlineStr">
         <is>
           <t>Energy is now conserved between turns.</t>
         </is>
@@ -25038,7 +25129,8 @@
       <c r="E91" t="n">
         <v>20</v>
       </c>
-      <c r="F91" t="inlineStr">
+      <c r="F91" t="inlineStr"/>
+      <c r="G91" t="inlineStr">
         <is>
           <t>Upon pickup, Transform a starter card with an ancient version.</t>
         </is>
@@ -25064,7 +25156,8 @@
       <c r="E92" t="n">
         <v>25</v>
       </c>
-      <c r="F92" t="inlineStr">
+      <c r="F92" t="inlineStr"/>
+      <c r="G92" t="inlineStr">
         <is>
           <t>Upon pickup, gain 150 Gold.</t>
         </is>
@@ -25090,7 +25183,8 @@
       <c r="E93" t="n">
         <v>50</v>
       </c>
-      <c r="F93" t="inlineStr">
+      <c r="F93" t="inlineStr"/>
+      <c r="G93" t="inlineStr">
         <is>
           <t>If you do not play any Attacks during your turn, gain an additional [energy:1] next turn.</t>
         </is>
@@ -25116,7 +25210,8 @@
       <c r="E94" t="n">
         <v>75</v>
       </c>
-      <c r="F94" t="inlineStr">
+      <c r="F94" t="inlineStr"/>
+      <c r="G94" t="inlineStr">
         <is>
           <t>Upon pickup, add 1 Enthralled to your Deck.</t>
         </is>
@@ -25142,7 +25237,8 @@
       <c r="E95" t="n">
         <v>100</v>
       </c>
-      <c r="F95" t="inlineStr">
+      <c r="F95" t="inlineStr"/>
+      <c r="G95" t="inlineStr">
         <is>
           <t>Unknown</t>
         </is>
@@ -25168,7 +25264,8 @@
       <c r="E96" t="n">
         <v>75</v>
       </c>
-      <c r="F96" t="inlineStr">
+      <c r="F96" t="inlineStr"/>
+      <c r="G96" t="inlineStr">
         <is>
           <t>Gain 1 energy at the start of each turn.</t>
         </is>
@@ -25194,7 +25291,8 @@
       <c r="E97" t="n">
         <v>100</v>
       </c>
-      <c r="F97" t="inlineStr">
+      <c r="F97" t="inlineStr"/>
+      <c r="G97" t="inlineStr">
         <is>
           <t>Whenever you Exhaust a card, deal 1 damage to a random enemy.</t>
         </is>
@@ -25220,7 +25318,8 @@
       <c r="E98" t="n">
         <v>100</v>
       </c>
-      <c r="F98" t="inlineStr">
+      <c r="F98" t="inlineStr"/>
+      <c r="G98" t="inlineStr">
         <is>
           <t>At the start of each combat, Channel 1 Dark.</t>
         </is>
@@ -25246,7 +25345,8 @@
       <c r="E99" t="n">
         <v>100</v>
       </c>
-      <c r="F99" t="inlineStr">
+      <c r="F99" t="inlineStr"/>
+      <c r="G99" t="inlineStr">
         <is>
           <t>Upon pickup, remove 5 cards from your Deck.</t>
         </is>
@@ -25272,7 +25372,8 @@
       <c r="E100" t="n">
         <v>50</v>
       </c>
-      <c r="F100" t="inlineStr">
+      <c r="F100" t="inlineStr"/>
+      <c r="G100" t="inlineStr">
         <is>
           <t>Upon pickup, raise your Max HP by 14.</t>
         </is>
@@ -25298,7 +25399,8 @@
       <c r="E101" t="n">
         <v>100</v>
       </c>
-      <c r="F101" t="inlineStr">
+      <c r="F101" t="inlineStr"/>
+      <c r="G101" t="inlineStr">
         <is>
           <t>50% discount on all products!</t>
         </is>
@@ -25324,7 +25426,8 @@
       <c r="E102" t="n">
         <v>75</v>
       </c>
-      <c r="F102" t="inlineStr">
+      <c r="F102" t="inlineStr"/>
+      <c r="G102" t="inlineStr">
         <is>
           <t>Upon pickup, lose 15 HP and Upgrade 3 random cards.</t>
         </is>
@@ -25350,7 +25453,8 @@
       <c r="E103" t="n">
         <v>100</v>
       </c>
-      <c r="F103" t="inlineStr">
+      <c r="F103" t="inlineStr"/>
+      <c r="G103" t="inlineStr">
         <is>
           <t>Upon pickup, choose an Attack or Skill in your Deck to Enchant.</t>
         </is>
@@ -25376,7 +25480,8 @@
       <c r="E104" t="n">
         <v>50</v>
       </c>
-      <c r="F104" t="inlineStr">
+      <c r="F104" t="inlineStr"/>
+      <c r="G104" t="inlineStr">
         <is>
           <t>At the start of each combat, procure a Potion-Shaped Rock.</t>
         </is>
@@ -25402,7 +25507,8 @@
       <c r="E105" t="n">
         <v>75</v>
       </c>
-      <c r="F105" t="inlineStr">
+      <c r="F105" t="inlineStr"/>
+      <c r="G105" t="inlineStr">
         <is>
           <t>The merchant no longer runs out of cards, relics, or potions.</t>
         </is>
@@ -25428,7 +25534,8 @@
       <c r="E106" t="n">
         <v>0</v>
       </c>
-      <c r="F106" t="inlineStr">
+      <c r="F106" t="inlineStr"/>
+      <c r="G106" t="inlineStr">
         <is>
           <t>Upon pickup, remove 4 cards from your Deck.</t>
         </is>
@@ -25454,7 +25561,8 @@
       <c r="E107" t="n">
         <v>0</v>
       </c>
-      <c r="F107" t="inlineStr">
+      <c r="F107" t="inlineStr"/>
+      <c r="G107" t="inlineStr">
         <is>
           <t>At the start of your 3rd turn, gain 1 Strength and 1 Dexterity.</t>
         </is>
@@ -25480,7 +25588,8 @@
       <c r="E108" t="n">
         <v>50</v>
       </c>
-      <c r="F108" t="inlineStr">
+      <c r="F108" t="inlineStr"/>
+      <c r="G108" t="inlineStr">
         <is>
           <t>Transform ALL Strikes and Defends.</t>
         </is>
@@ -25506,7 +25615,8 @@
       <c r="E109" t="n">
         <v>66.7</v>
       </c>
-      <c r="F109" t="inlineStr">
+      <c r="F109" t="inlineStr"/>
+      <c r="G109" t="inlineStr">
         <is>
           <t>Every 5 times you Exhaust a card, draw 1 card.</t>
         </is>
@@ -25532,7 +25642,8 @@
       <c r="E110" t="n">
         <v>100</v>
       </c>
-      <c r="F110" t="inlineStr">
+      <c r="F110" t="inlineStr"/>
+      <c r="G110" t="inlineStr">
         <is>
           <t>Upon pickup, raise your Max HP by 31.</t>
         </is>
@@ -25558,7 +25669,8 @@
       <c r="E111" t="n">
         <v>100</v>
       </c>
-      <c r="F111" t="inlineStr">
+      <c r="F111" t="inlineStr"/>
+      <c r="G111" t="inlineStr">
         <is>
           <t>Whenever you play a card that costs 2 or more, gain 4 Block.</t>
         </is>
@@ -25584,7 +25696,8 @@
       <c r="E112" t="n">
         <v>66.7</v>
       </c>
-      <c r="F112" t="inlineStr">
+      <c r="F112" t="inlineStr"/>
+      <c r="G112" t="inlineStr">
         <is>
           <t>At the end of turn 7, deal 52 damage to ALL enemies.</t>
         </is>
@@ -25610,7 +25723,8 @@
       <c r="E113" t="n">
         <v>66.7</v>
       </c>
-      <c r="F113" t="inlineStr">
+      <c r="F113" t="inlineStr"/>
+      <c r="G113" t="inlineStr">
         <is>
           <t>Unknown</t>
         </is>
@@ -25636,7 +25750,8 @@
       <c r="E114" t="n">
         <v>33.3</v>
       </c>
-      <c r="F114" t="inlineStr">
+      <c r="F114" t="inlineStr"/>
+      <c r="G114" t="inlineStr">
         <is>
           <t>Upon pickup, obtain a random Relic.</t>
         </is>
@@ -25662,7 +25777,8 @@
       <c r="E115" t="n">
         <v>66.7</v>
       </c>
-      <c r="F115" t="inlineStr">
+      <c r="F115" t="inlineStr"/>
+      <c r="G115" t="inlineStr">
         <is>
           <t>Whenever you lose HP in combat, gain 3 Block next turn.</t>
         </is>
@@ -25688,7 +25804,8 @@
       <c r="E116" t="n">
         <v>66.7</v>
       </c>
-      <c r="F116" t="inlineStr">
+      <c r="F116" t="inlineStr"/>
+      <c r="G116" t="inlineStr">
         <is>
           <t>You may Cook at Rest Sites.</t>
         </is>
@@ -25714,7 +25831,8 @@
       <c r="E117" t="n">
         <v>33.3</v>
       </c>
-      <c r="F117" t="inlineStr">
+      <c r="F117" t="inlineStr"/>
+      <c r="G117" t="inlineStr">
         <is>
           <t>Whenever you add an Attack card to your Deck, Upgrade it.</t>
         </is>
@@ -25740,7 +25858,8 @@
       <c r="E118" t="n">
         <v>33.3</v>
       </c>
-      <c r="F118" t="inlineStr">
+      <c r="F118" t="inlineStr"/>
+      <c r="G118" t="inlineStr">
         <is>
           <t>Whenever you kill an Elite, Upgrade 4 random cards.</t>
         </is>
@@ -25766,7 +25885,8 @@
       <c r="E119" t="n">
         <v>33.3</v>
       </c>
-      <c r="F119" t="inlineStr">
+      <c r="F119" t="inlineStr"/>
+      <c r="G119" t="inlineStr">
         <is>
           <t>Upon pickup, remove 5 cards from your Deck.</t>
         </is>
@@ -25792,7 +25912,8 @@
       <c r="E120" t="n">
         <v>33.3</v>
       </c>
-      <c r="F120" t="inlineStr">
+      <c r="F120" t="inlineStr"/>
+      <c r="G120" t="inlineStr">
         <is>
           <t>At the start of each combat, apply 4 Poison to ALL enemies.</t>
         </is>
@@ -25818,7 +25939,8 @@
       <c r="E121" t="n">
         <v>66.7</v>
       </c>
-      <c r="F121" t="inlineStr">
+      <c r="F121" t="inlineStr"/>
+      <c r="G121" t="inlineStr">
         <is>
           <t>At the start of your turn, deal damage equal to the turn number to ALL enemies.</t>
         </is>
@@ -25844,7 +25966,8 @@
       <c r="E122" t="n">
         <v>66.7</v>
       </c>
-      <c r="F122" t="inlineStr">
+      <c r="F122" t="inlineStr"/>
+      <c r="G122" t="inlineStr">
         <is>
           <t>Whenever you play 3 or fewer cards during your turn, draw 3 additional cards.</t>
         </is>
@@ -25870,7 +25993,8 @@
       <c r="E123" t="n">
         <v>33.3</v>
       </c>
-      <c r="F123" t="inlineStr">
+      <c r="F123" t="inlineStr"/>
+      <c r="G123" t="inlineStr">
         <is>
           <t>Upon pickup, gain 1 card reward and procure 1 random potion.</t>
         </is>
@@ -25896,7 +26020,8 @@
       <c r="E124" t="n">
         <v>66.7</v>
       </c>
-      <c r="F124" t="inlineStr">
+      <c r="F124" t="inlineStr"/>
+      <c r="G124" t="inlineStr">
         <is>
           <t>At the start of the next combat, Upgrade your starting hand.</t>
         </is>
@@ -25922,7 +26047,8 @@
       <c r="E125" t="n">
         <v>66.7</v>
       </c>
-      <c r="F125" t="inlineStr">
+      <c r="F125" t="inlineStr"/>
+      <c r="G125" t="inlineStr">
         <is>
           <t>The first time you Channel 7 Orbs each combat, deal 30 damage to ALL enemies.</t>
         </is>
@@ -25948,7 +26074,8 @@
       <c r="E126" t="n">
         <v>66.7</v>
       </c>
-      <c r="F126" t="inlineStr">
+      <c r="F126" t="inlineStr"/>
+      <c r="G126" t="inlineStr">
         <is>
           <t>At the start of each combat, add 1 of 5 random cards into your Hand.</t>
         </is>
@@ -25974,7 +26101,8 @@
       <c r="E127" t="n">
         <v>33.3</v>
       </c>
-      <c r="F127" t="inlineStr">
+      <c r="F127" t="inlineStr"/>
+      <c r="G127" t="inlineStr">
         <is>
           <t>Upon pickup, obtain 2 Common cards, 2 Uncommon cards, and 1 Rare card.</t>
         </is>
@@ -26000,7 +26128,8 @@
       <c r="E128" t="n">
         <v>0</v>
       </c>
-      <c r="F128" t="inlineStr">
+      <c r="F128" t="inlineStr"/>
+      <c r="G128" t="inlineStr">
         <is>
           <t>Upon pickup, Upgrade 6 random cards.</t>
         </is>
@@ -26026,7 +26155,8 @@
       <c r="E129" t="n">
         <v>50</v>
       </c>
-      <c r="F129" t="inlineStr">
+      <c r="F129" t="inlineStr"/>
+      <c r="G129" t="inlineStr">
         <is>
           <t>Upon pickup, add 1 Whistle to your Deck.</t>
         </is>
@@ -26052,7 +26182,8 @@
       <c r="E130" t="n">
         <v>50</v>
       </c>
-      <c r="F130" t="inlineStr">
+      <c r="F130" t="inlineStr"/>
+      <c r="G130" t="inlineStr">
         <is>
           <t>Whenever you add a Skill into your Deck, Upgrade it.</t>
         </is>
@@ -26078,7 +26209,8 @@
       <c r="E131" t="n">
         <v>50</v>
       </c>
-      <c r="F131" t="inlineStr">
+      <c r="F131" t="inlineStr"/>
+      <c r="G131" t="inlineStr">
         <is>
           <t>Every time you play 3 Attacks in a single turn, gain 1 Dexterity.</t>
         </is>
@@ -26104,7 +26236,8 @@
       <c r="E132" t="n">
         <v>100</v>
       </c>
-      <c r="F132" t="inlineStr">
+      <c r="F132" t="inlineStr"/>
+      <c r="G132" t="inlineStr">
         <is>
           <t>At the end of your turn, you no longer discard your Hand.</t>
         </is>
@@ -26130,7 +26263,8 @@
       <c r="E133" t="n">
         <v>50</v>
       </c>
-      <c r="F133" t="inlineStr">
+      <c r="F133" t="inlineStr"/>
+      <c r="G133" t="inlineStr">
         <is>
           <t>Whenever you add a card to your Deck, add one additional copy.</t>
         </is>
@@ -26156,7 +26290,8 @@
       <c r="E134" t="n">
         <v>50</v>
       </c>
-      <c r="F134" t="inlineStr">
+      <c r="F134" t="inlineStr"/>
+      <c r="G134" t="inlineStr">
         <is>
           <t>Elites drop an additional Rare card reward.</t>
         </is>
@@ -26182,7 +26317,8 @@
       <c r="E135" t="n">
         <v>100</v>
       </c>
-      <c r="F135" t="inlineStr">
+      <c r="F135" t="inlineStr"/>
+      <c r="G135" t="inlineStr">
         <is>
           <t>At the start of your turn, draw 1 additional card.</t>
         </is>
@@ -26208,7 +26344,8 @@
       <c r="E136" t="n">
         <v>100</v>
       </c>
-      <c r="F136" t="inlineStr">
+      <c r="F136" t="inlineStr"/>
+      <c r="G136" t="inlineStr">
         <is>
           <t>Upon pickup, gain 5 card rewards.</t>
         </is>
@@ -26234,7 +26371,8 @@
       <c r="E137" t="n">
         <v>100</v>
       </c>
-      <c r="F137" t="inlineStr">
+      <c r="F137" t="inlineStr"/>
+      <c r="G137" t="inlineStr">
         <is>
           <t>Potions always appear in combat rewards.</t>
         </is>
@@ -26260,7 +26398,8 @@
       <c r="E138" t="n">
         <v>100</v>
       </c>
-      <c r="F138" t="inlineStr">
+      <c r="F138" t="inlineStr"/>
+      <c r="G138" t="inlineStr">
         <is>
           <t>Enemies with Vulnerable take 75% more damage.</t>
         </is>
@@ -26286,7 +26425,8 @@
       <c r="E139" t="n">
         <v>100</v>
       </c>
-      <c r="F139" t="inlineStr">
+      <c r="F139" t="inlineStr"/>
+      <c r="G139" t="inlineStr">
         <is>
           <t>Strikes and Defends gain Ethereal.</t>
         </is>
@@ -26312,7 +26452,8 @@
       <c r="E140" t="n">
         <v>100</v>
       </c>
-      <c r="F140" t="inlineStr">
+      <c r="F140" t="inlineStr"/>
+      <c r="G140" t="inlineStr">
         <is>
           <t>Whenever you apply Poison, apply an additional 1 Poison.</t>
         </is>
@@ -26338,7 +26479,8 @@
       <c r="E141" t="n">
         <v>50</v>
       </c>
-      <c r="F141" t="inlineStr">
+      <c r="F141" t="inlineStr"/>
+      <c r="G141" t="inlineStr">
         <is>
           <t>Gain 1 energy at the start of each turn. Card rewards contain cards from other colors.</t>
         </is>
@@ -26364,7 +26506,8 @@
       <c r="E142" t="n">
         <v>100</v>
       </c>
-      <c r="F142" t="inlineStr">
+      <c r="F142" t="inlineStr"/>
+      <c r="G142" t="inlineStr">
         <is>
           <t>Upon pickup, choose 3 cards in your Deck. Enchant them with [purple]Swift[/purple] 3.</t>
         </is>
@@ -26390,7 +26533,8 @@
       <c r="E143" t="n">
         <v>100</v>
       </c>
-      <c r="F143" t="inlineStr">
+      <c r="F143" t="inlineStr"/>
+      <c r="G143" t="inlineStr">
         <is>
           <t>Enchant all card rewards with Glam.</t>
         </is>
@@ -26416,7 +26560,8 @@
       <c r="E144" t="n">
         <v>50</v>
       </c>
-      <c r="F144" t="inlineStr">
+      <c r="F144" t="inlineStr"/>
+      <c r="G144" t="inlineStr">
         <is>
           <t>You can now dig at Rest Sites to obtain a random Relic.</t>
         </is>
@@ -26442,7 +26587,8 @@
       <c r="E145" t="n">
         <v>50</v>
       </c>
-      <c r="F145" t="inlineStr">
+      <c r="F145" t="inlineStr"/>
+      <c r="G145" t="inlineStr">
         <is>
           <t>Whenever you discard a card during your turn, deal 3 damage to a random enemy.</t>
         </is>
@@ -26468,7 +26614,8 @@
       <c r="E146" t="n">
         <v>100</v>
       </c>
-      <c r="F146" t="inlineStr">
+      <c r="F146" t="inlineStr"/>
+      <c r="G146" t="inlineStr">
         <is>
           <t>Upon pickup, replace your starter Relic with an Ancient version.</t>
         </is>
@@ -26494,7 +26641,8 @@
       <c r="E147" t="n">
         <v>0</v>
       </c>
-      <c r="F147" t="inlineStr">
+      <c r="F147" t="inlineStr"/>
+      <c r="G147" t="inlineStr">
         <is>
           <t>At the start of the next 5 combats, gain 2 Strength.</t>
         </is>
@@ -26520,7 +26668,8 @@
       <c r="E148" t="n">
         <v>0</v>
       </c>
-      <c r="F148" t="inlineStr">
+      <c r="F148" t="inlineStr"/>
+      <c r="G148" t="inlineStr">
         <is>
           <t>You can now gain Strength at Rest Sites. (3 times max)</t>
         </is>
@@ -26546,7 +26695,8 @@
       <c r="E149" t="n">
         <v>100</v>
       </c>
-      <c r="F149" t="inlineStr">
+      <c r="F149" t="inlineStr"/>
+      <c r="G149" t="inlineStr">
         <is>
           <t>Unknown</t>
         </is>
@@ -26572,7 +26722,8 @@
       <c r="E150" t="n">
         <v>0</v>
       </c>
-      <c r="F150" t="inlineStr">
+      <c r="F150" t="inlineStr"/>
+      <c r="G150" t="inlineStr">
         <is>
           <t>Upon pickup, add 1 Neow's Fury to your Deck.</t>
         </is>
@@ -26598,7 +26749,8 @@
       <c r="E151" t="n">
         <v>0</v>
       </c>
-      <c r="F151" t="inlineStr">
+      <c r="F151" t="inlineStr"/>
+      <c r="G151" t="inlineStr">
         <is>
           <t>Upon pickup, add 1 Apotheosis to your Deck.</t>
         </is>
@@ -26624,7 +26776,8 @@
       <c r="E152" t="n">
         <v>50</v>
       </c>
-      <c r="F152" t="inlineStr">
+      <c r="F152" t="inlineStr"/>
+      <c r="G152" t="inlineStr">
         <is>
           <t>At the start of each combat, discard any number of cards then draw that many.</t>
         </is>
@@ -26650,7 +26803,8 @@
       <c r="E153" t="n">
         <v>50</v>
       </c>
-      <c r="F153" t="inlineStr">
+      <c r="F153" t="inlineStr"/>
+      <c r="G153" t="inlineStr">
         <is>
           <t>If you end your turn with unspent energy, gain additional energy next turn.</t>
         </is>
@@ -26676,7 +26830,8 @@
       <c r="E154" t="n">
         <v>100</v>
       </c>
-      <c r="F154" t="inlineStr">
+      <c r="F154" t="inlineStr"/>
+      <c r="G154" t="inlineStr">
         <is>
           <t>At the start of your turn, draw 2 additional cards.</t>
         </is>
@@ -26702,7 +26857,8 @@
       <c r="E155" t="n">
         <v>50</v>
       </c>
-      <c r="F155" t="inlineStr">
+      <c r="F155" t="inlineStr"/>
+      <c r="G155" t="inlineStr">
         <is>
           <t>Upon pickup, Enchant a card with Clone.</t>
         </is>
@@ -26728,7 +26884,8 @@
       <c r="E156" t="n">
         <v>50</v>
       </c>
-      <c r="F156" t="inlineStr">
+      <c r="F156" t="inlineStr"/>
+      <c r="G156" t="inlineStr">
         <is>
           <t>Whenever you have no cards in Hand during your turn, draw a card.</t>
         </is>
@@ -26754,7 +26911,8 @@
       <c r="E157" t="n">
         <v>100</v>
       </c>
-      <c r="F157" t="inlineStr">
+      <c r="F157" t="inlineStr"/>
+      <c r="G157" t="inlineStr">
         <is>
           <t>Every 4 cards you play, draw 1 card.</t>
         </is>
@@ -26780,7 +26938,8 @@
       <c r="E158" t="n">
         <v>50</v>
       </c>
-      <c r="F158" t="inlineStr">
+      <c r="F158" t="inlineStr"/>
+      <c r="G158" t="inlineStr">
         <is>
           <t>Upon pickup, obtain an additional copy of a card in your Deck.</t>
         </is>
@@ -26806,7 +26965,8 @@
       <c r="E159" t="n">
         <v>0</v>
       </c>
-      <c r="F159" t="inlineStr">
+      <c r="F159" t="inlineStr"/>
+      <c r="G159" t="inlineStr">
         <is>
           <t>Upon pickup, gain 4 potion slots filled with random potions.</t>
         </is>
@@ -26832,7 +26992,8 @@
       <c r="E160" t="n">
         <v>0</v>
       </c>
-      <c r="F160" t="inlineStr">
+      <c r="F160" t="inlineStr"/>
+      <c r="G160" t="inlineStr">
         <is>
           <t>Transforms into a powerful Relic after defeating 5 Elites.</t>
         </is>
@@ -26858,7 +27019,8 @@
       <c r="E161" t="n">
         <v>100</v>
       </c>
-      <c r="F161" t="inlineStr">
+      <c r="F161" t="inlineStr"/>
+      <c r="G161" t="inlineStr">
         <is>
           <t>Unknown</t>
         </is>
@@ -26884,7 +27046,8 @@
       <c r="E162" t="n">
         <v>100</v>
       </c>
-      <c r="F162" t="inlineStr">
+      <c r="F162" t="inlineStr"/>
+      <c r="G162" t="inlineStr">
         <is>
           <t>You may sacrifice card rewards to Pael.</t>
         </is>
@@ -26910,7 +27073,8 @@
       <c r="E163" t="n">
         <v>100</v>
       </c>
-      <c r="F163" t="inlineStr">
+      <c r="F163" t="inlineStr"/>
+      <c r="G163" t="inlineStr">
         <is>
           <t>Unknown</t>
         </is>
@@ -26936,7 +27100,8 @@
       <c r="E164" t="n">
         <v>0</v>
       </c>
-      <c r="F164" t="inlineStr">
+      <c r="F164" t="inlineStr"/>
+      <c r="G164" t="inlineStr">
         <is>
           <t>See 15 cards from another character.</t>
         </is>
@@ -26962,7 +27127,8 @@
       <c r="E165" t="n">
         <v>100</v>
       </c>
-      <c r="F165" t="inlineStr">
+      <c r="F165" t="inlineStr"/>
+      <c r="G165" t="inlineStr">
         <is>
           <t>Upon pickup, gain the card Byrd Swoop.</t>
         </is>
@@ -26988,7 +27154,8 @@
       <c r="E166" t="n">
         <v>100</v>
       </c>
-      <c r="F166" t="inlineStr">
+      <c r="F166" t="inlineStr"/>
+      <c r="G166" t="inlineStr">
         <is>
           <t>Upon pickup, add 2 Relax to your Deck.</t>
         </is>
@@ -27014,7 +27181,8 @@
       <c r="E167" t="n">
         <v>100</v>
       </c>
-      <c r="F167" t="inlineStr">
+      <c r="F167" t="inlineStr"/>
+      <c r="G167" t="inlineStr">
         <is>
           <t>Upon pickup, Transform up to 6 cards into Maul.</t>
         </is>
@@ -27040,7 +27208,8 @@
       <c r="E168" t="n">
         <v>100</v>
       </c>
-      <c r="F168" t="inlineStr">
+      <c r="F168" t="inlineStr"/>
+      <c r="G168" t="inlineStr">
         <is>
           <t>Unknown</t>
         </is>
@@ -27066,7 +27235,8 @@
       <c r="E169" t="n">
         <v>100</v>
       </c>
-      <c r="F169" t="inlineStr">
+      <c r="F169" t="inlineStr"/>
+      <c r="G169" t="inlineStr">
         <is>
           <t>Unknown</t>
         </is>
@@ -27092,7 +27262,8 @@
       <c r="E170" t="n">
         <v>100</v>
       </c>
-      <c r="F170" t="inlineStr">
+      <c r="F170" t="inlineStr"/>
+      <c r="G170" t="inlineStr">
         <is>
           <t>At the start of each combat, add 3 Souls into your Draw Pile.</t>
         </is>
@@ -27118,7 +27289,8 @@
       <c r="E171" t="n">
         <v>100</v>
       </c>
-      <c r="F171" t="inlineStr">
+      <c r="F171" t="inlineStr"/>
+      <c r="G171" t="inlineStr">
         <is>
           <t>Upon pickup, obtain 4 Wax Relics.</t>
         </is>
@@ -27144,7 +27316,8 @@
       <c r="E172" t="n">
         <v>100</v>
       </c>
-      <c r="F172" t="inlineStr">
+      <c r="F172" t="inlineStr"/>
+      <c r="G172" t="inlineStr">
         <is>
           <t>Start each combat with 3 additional Orb Slots.</t>
         </is>
@@ -27170,7 +27343,8 @@
       <c r="E173" t="n">
         <v>0</v>
       </c>
-      <c r="F173" t="inlineStr">
+      <c r="F173" t="inlineStr"/>
+      <c r="G173" t="inlineStr">
         <is>
           <t>Upon pickup, Transform 3 cards, then Upgrade them.</t>
         </is>
@@ -27196,7 +27370,8 @@
       <c r="E174" t="n">
         <v>100</v>
       </c>
-      <c r="F174" t="inlineStr">
+      <c r="F174" t="inlineStr"/>
+      <c r="G174" t="inlineStr">
         <is>
           <t>Whenever you shuffle your Draw Pile, gain 6 Block.</t>
         </is>
@@ -27222,7 +27397,8 @@
       <c r="E175" t="n">
         <v>0</v>
       </c>
-      <c r="F175" t="inlineStr">
+      <c r="F175" t="inlineStr"/>
+      <c r="G175" t="inlineStr">
         <is>
           <t>You may reroll each card reward once.</t>
         </is>
@@ -27248,7 +27424,8 @@
       <c r="E176" t="n">
         <v>0</v>
       </c>
-      <c r="F176" t="inlineStr">
+      <c r="F176" t="inlineStr"/>
+      <c r="G176" t="inlineStr">
         <is>
           <t>Gain an additional energy at the start of your 3rd turn.</t>
         </is>
@@ -27274,7 +27451,8 @@
       <c r="E177" t="n">
         <v>0</v>
       </c>
-      <c r="F177" t="inlineStr">
+      <c r="F177" t="inlineStr"/>
+      <c r="G177" t="inlineStr">
         <is>
           <t>Whenever you create a Colorless card, gain 2 Block.</t>
         </is>
@@ -27300,7 +27478,8 @@
       <c r="E178" t="n">
         <v>0</v>
       </c>
-      <c r="F178" t="inlineStr">
+      <c r="F178" t="inlineStr"/>
+      <c r="G178" t="inlineStr">
         <is>
           <t>Enchanted Attacks deal 9 additional damage.</t>
         </is>
@@ -27326,7 +27505,8 @@
       <c r="E179" t="n">
         <v>100</v>
       </c>
-      <c r="F179" t="inlineStr">
+      <c r="F179" t="inlineStr"/>
+      <c r="G179" t="inlineStr">
         <is>
           <t>Upon pickup, raise your Max HP by 11.</t>
         </is>
@@ -27352,7 +27532,8 @@
       <c r="E180" t="n">
         <v>100</v>
       </c>
-      <c r="F180" t="inlineStr">
+      <c r="F180" t="inlineStr"/>
+      <c r="G180" t="inlineStr">
         <is>
           <t>Upon pickup, add 1 Brightest Flame to your Deck.</t>
         </is>
@@ -27378,7 +27559,8 @@
       <c r="E181" t="n">
         <v>100</v>
       </c>
-      <c r="F181" t="inlineStr">
+      <c r="F181" t="inlineStr"/>
+      <c r="G181" t="inlineStr">
         <is>
           <t>The effects of your cost X cards are increased by 2.</t>
         </is>
@@ -27404,7 +27586,8 @@
       <c r="E182" t="n">
         <v>100</v>
       </c>
-      <c r="F182" t="inlineStr">
+      <c r="F182" t="inlineStr"/>
+      <c r="G182" t="inlineStr">
         <is>
           <t>At the start of each combat, add 2 random Ethereal cards into your Hand.</t>
         </is>
@@ -27430,7 +27613,8 @@
       <c r="E183" t="n">
         <v>100</v>
       </c>
-      <c r="F183" t="inlineStr">
+      <c r="F183" t="inlineStr"/>
+      <c r="G183" t="inlineStr">
         <is>
           <t>Upon pickup, gain 300 Gold.</t>
         </is>
@@ -27456,7 +27640,8 @@
       <c r="E184" t="n">
         <v>100</v>
       </c>
-      <c r="F184" t="inlineStr">
+      <c r="F184" t="inlineStr"/>
+      <c r="G184" t="inlineStr">
         <is>
           <t>Every time you play an Attack or Skill, Upgrade it for the remainder of combat.</t>
         </is>
@@ -27482,7 +27667,8 @@
       <c r="E185" t="n">
         <v>100</v>
       </c>
-      <c r="F185" t="inlineStr">
+      <c r="F185" t="inlineStr"/>
+      <c r="G185" t="inlineStr">
         <is>
           <t>Enemies with Weak deal 40% less damage to you.</t>
         </is>
@@ -27508,7 +27694,8 @@
       <c r="E186" t="n">
         <v>100</v>
       </c>
-      <c r="F186" t="inlineStr">
+      <c r="F186" t="inlineStr"/>
+      <c r="G186" t="inlineStr">
         <is>
           <t>A random card in each card reward is Enchanted with Swift 1.</t>
         </is>
@@ -27534,7 +27721,8 @@
       <c r="E187" t="n">
         <v>0</v>
       </c>
-      <c r="F187" t="inlineStr">
+      <c r="F187" t="inlineStr"/>
+      <c r="G187" t="inlineStr">
         <is>
           <t>Upon pickup, Enchant all Strikes in your Deck.</t>
         </is>
@@ -27560,7 +27748,8 @@
       <c r="E188" t="n">
         <v>0</v>
       </c>
-      <c r="F188" t="inlineStr">
+      <c r="F188" t="inlineStr"/>
+      <c r="G188" t="inlineStr">
         <is>
           <t>Whenever you gain Gold, raise your Max HP by 1.</t>
         </is>
@@ -27586,7 +27775,8 @@
       <c r="E189" t="n">
         <v>100</v>
       </c>
-      <c r="F189" t="inlineStr">
+      <c r="F189" t="inlineStr"/>
+      <c r="G189" t="inlineStr">
         <is>
           <t>At the start of each combat, Summon 5. At the start of your turn, Summon 2.</t>
         </is>
@@ -27612,7 +27802,8 @@
       <c r="E190" t="n">
         <v>0</v>
       </c>
-      <c r="F190" t="inlineStr">
+      <c r="F190" t="inlineStr"/>
+      <c r="G190" t="inlineStr">
         <is>
           <t>Upon pickup, Enchant up to 3 cards with Adroit.</t>
         </is>
@@ -27638,7 +27829,8 @@
       <c r="E191" t="n">
         <v>100</v>
       </c>
-      <c r="F191" t="inlineStr">
+      <c r="F191" t="inlineStr"/>
+      <c r="G191" t="inlineStr">
         <is>
           <t>Upon pickup, choose 1 of 3 Multiplayer Cards to add to your Deck.</t>
         </is>
@@ -27664,7 +27856,8 @@
       <c r="E192" t="n">
         <v>100</v>
       </c>
-      <c r="F192" t="inlineStr">
+      <c r="F192" t="inlineStr"/>
+      <c r="G192" t="inlineStr">
         <is>
           <t>The first time each combat you Exhaust a Skill, add a copy of it into your Hand.</t>
         </is>
@@ -27690,7 +27883,8 @@
       <c r="E193" t="n">
         <v>0</v>
       </c>
-      <c r="F193" t="inlineStr">
+      <c r="F193" t="inlineStr"/>
+      <c r="G193" t="inlineStr">
         <is>
           <t>Upon pickup, Enchant a Skill with Imbued.</t>
         </is>
@@ -27716,7 +27910,8 @@
       <c r="E194" t="n">
         <v>100</v>
       </c>
-      <c r="F194" t="inlineStr">
+      <c r="F194" t="inlineStr"/>
+      <c r="G194" t="inlineStr">
         <is>
           <t>Unknown</t>
         </is>
@@ -27742,7 +27937,8 @@
       <c r="E195" t="n">
         <v>0</v>
       </c>
-      <c r="F195" t="inlineStr">
+      <c r="F195" t="inlineStr"/>
+      <c r="G195" t="inlineStr">
         <is>
           <t>At the start of each combat, add 2 zero-cost cards from your Draw Pile into your Hand.</t>
         </is>
@@ -27768,7 +27964,8 @@
       <c r="E196" t="n">
         <v>0</v>
       </c>
-      <c r="F196" t="inlineStr">
+      <c r="F196" t="inlineStr"/>
+      <c r="G196" t="inlineStr">
         <is>
           <t>Whenever you play a Power, deal 8 damage to ALL enemies.</t>
         </is>
@@ -27794,7 +27991,8 @@
       <c r="E197" t="n">
         <v>0</v>
       </c>
-      <c r="F197" t="inlineStr">
+      <c r="F197" t="inlineStr"/>
+      <c r="G197" t="inlineStr">
         <is>
           <t>Upon pickup, lose 9 Max HP. Add 3 Apparitions to your Deck.</t>
         </is>
@@ -27820,7 +28018,8 @@
       <c r="E198" t="n">
         <v>0</v>
       </c>
-      <c r="F198" t="inlineStr">
+      <c r="F198" t="inlineStr"/>
+      <c r="G198" t="inlineStr">
         <is>
           <t>Every other combat, your card rewards gain an additional Power.</t>
         </is>
@@ -27846,7 +28045,8 @@
       <c r="E199" t="n">
         <v>100</v>
       </c>
-      <c r="F199" t="inlineStr">
+      <c r="F199" t="inlineStr"/>
+      <c r="G199" t="inlineStr">
         <is>
           <t>At the start of each combat, add a random card into your Hand.</t>
         </is>
@@ -27872,7 +28072,8 @@
       <c r="E200" t="n">
         <v>100</v>
       </c>
-      <c r="F200" t="inlineStr">
+      <c r="F200" t="inlineStr"/>
+      <c r="G200" t="inlineStr">
         <is>
           <t>Whenever you play an Attack, gain 1 Block.</t>
         </is>
@@ -27898,7 +28099,8 @@
       <c r="E201" t="n">
         <v>0</v>
       </c>
-      <c r="F201" t="inlineStr">
+      <c r="F201" t="inlineStr"/>
+      <c r="G201" t="inlineStr">
         <is>
           <t>Whenever you break an enemy's Block, apply 2 Vulnerable.</t>
         </is>
@@ -27924,7 +28126,8 @@
       <c r="E202" t="n">
         <v>100</v>
       </c>
-      <c r="F202" t="inlineStr">
+      <c r="F202" t="inlineStr"/>
+      <c r="G202" t="inlineStr">
         <is>
           <t>At the start of your first turn, lose 2 energy.</t>
         </is>
@@ -27950,7 +28153,8 @@
       <c r="E203" t="n">
         <v>100</v>
       </c>
-      <c r="F203" t="inlineStr">
+      <c r="F203" t="inlineStr"/>
+      <c r="G203" t="inlineStr">
         <is>
           <t>The first time you spend Star each turn, gain 1 Strength.</t>
         </is>
@@ -27976,7 +28180,8 @@
       <c r="E204" t="n">
         <v>100</v>
       </c>
-      <c r="F204" t="inlineStr">
+      <c r="F204" t="inlineStr"/>
+      <c r="G204" t="inlineStr">
         <is>
           <t>Start each combat with 3 Strength.</t>
         </is>
@@ -28002,7 +28207,8 @@
       <c r="E205" t="n">
         <v>100</v>
       </c>
-      <c r="F205" t="inlineStr">
+      <c r="F205" t="inlineStr"/>
+      <c r="G205" t="inlineStr">
         <is>
           <t>Upgraded Attacks deal 3 additional damage.</t>
         </is>
@@ -28028,7 +28234,8 @@
       <c r="E206" t="n">
         <v>100</v>
       </c>
-      <c r="F206" t="inlineStr">
+      <c r="F206" t="inlineStr"/>
+      <c r="G206" t="inlineStr">
         <is>
           <t>The first time you gain Strength each combat, double the amount gained.</t>
         </is>
@@ -28054,7 +28261,8 @@
       <c r="E207" t="n">
         <v>100</v>
       </c>
-      <c r="F207" t="inlineStr">
+      <c r="F207" t="inlineStr"/>
+      <c r="G207" t="inlineStr">
         <is>
           <t>At the start of your turn, play a copy of your last played Attack or Skill.</t>
         </is>
@@ -28080,7 +28288,8 @@
       <c r="E208" t="n">
         <v>100</v>
       </c>
-      <c r="F208" t="inlineStr">
+      <c r="F208" t="inlineStr"/>
+      <c r="G208" t="inlineStr">
         <is>
           <t>Retain your Hand on the first turn of combat.</t>
         </is>
@@ -28106,7 +28315,8 @@
       <c r="E209" t="n">
         <v>0</v>
       </c>
-      <c r="F209" t="inlineStr">
+      <c r="F209" t="inlineStr"/>
+      <c r="G209" t="inlineStr">
         <is>
           <t>At the start of Elite combats, draw 2 additional cards.</t>
         </is>
@@ -28132,7 +28342,8 @@
       <c r="E210" t="n">
         <v>0</v>
       </c>
-      <c r="F210" t="inlineStr">
+      <c r="F210" t="inlineStr"/>
+      <c r="G210" t="inlineStr">
         <is>
           <t>At the start of the next combat, shuffle 2 Dazed into your Draw Pile.</t>
         </is>
@@ -28158,7 +28369,8 @@
       <c r="E211" t="n">
         <v>0</v>
       </c>
-      <c r="F211" t="inlineStr">
+      <c r="F211" t="inlineStr"/>
+      <c r="G211" t="inlineStr">
         <is>
           <t>Upon pickup, mark 7 random combats.</t>
         </is>
@@ -28184,7 +28396,8 @@
       <c r="E212" t="n">
         <v>100</v>
       </c>
-      <c r="F212" t="inlineStr">
+      <c r="F212" t="inlineStr"/>
+      <c r="G212" t="inlineStr">
         <is>
           <t>Upon pickup, raise your Max HP by 7 and heal all of your HP.</t>
         </is>
@@ -28210,7 +28423,8 @@
       <c r="E213" t="n">
         <v>0</v>
       </c>
-      <c r="F213" t="inlineStr">
+      <c r="F213" t="inlineStr"/>
+      <c r="G213" t="inlineStr">
         <is>
           <t>At the start of your turn, Exhaust the top card of your Draw Pile and gain 1 Strength.</t>
         </is>
@@ -28236,7 +28450,8 @@
       <c r="E214" t="n">
         <v>100</v>
       </c>
-      <c r="F214" t="inlineStr">
+      <c r="F214" t="inlineStr"/>
+      <c r="G214" t="inlineStr">
         <is>
           <t>At the start of each combat, Channel 3 Lightning.</t>
         </is>
@@ -28262,7 +28477,8 @@
       <c r="E215" t="n">
         <v>100</v>
       </c>
-      <c r="F215" t="inlineStr">
+      <c r="F215" t="inlineStr"/>
+      <c r="G215" t="inlineStr">
         <is>
           <t>Your rightmost Orb triggers its passive an additional time.</t>
         </is>
@@ -28288,7 +28504,8 @@
       <c r="E216" t="n">
         <v>100</v>
       </c>
-      <c r="F216" t="inlineStr">
+      <c r="F216" t="inlineStr"/>
+      <c r="G216" t="inlineStr">
         <is>
           <t>Every 4 turns, draw 2 additional cards.</t>
         </is>
@@ -28314,7 +28531,8 @@
       <c r="E217" t="n">
         <v>0</v>
       </c>
-      <c r="F217" t="inlineStr">
+      <c r="F217" t="inlineStr"/>
+      <c r="G217" t="inlineStr">
         <is>
           <t>Whenever you obtain a Curse, raise your Max HP by 6.</t>
         </is>
@@ -28340,7 +28558,8 @@
       <c r="E218" t="n">
         <v>0</v>
       </c>
-      <c r="F218" t="inlineStr">
+      <c r="F218" t="inlineStr"/>
+      <c r="G218" t="inlineStr">
         <is>
           <t>Upon pickup, obtain a unique Curse and 3 Relics.</t>
         </is>

</xml_diff>